<commit_message>
Update binary files for Body Masters and Body Motions reports
</commit_message>
<xml_diff>
--- a/Month YEAR - Body Motions.xlsx
+++ b/Month YEAR - Body Motions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andyayas/VALD Automator/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D341DE7-1F84-1B4C-9446-D521A65A3CF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{414C0AF1-7EE3-BD45-AC8A-E8B524C6DAB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,8 +34,8 @@
     <sheet name="Tabuk" sheetId="20" r:id="rId19"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">REPORT!$B$1:$B$322</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">REPORT!$A$1:$D$176</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">REPORT!$B$1:$B$323</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">REPORT!$A$1:$D$177</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'REPORT 2'!$A$1:$G$14</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'REPORT 2'!$1:$6</definedName>
   </definedNames>
@@ -82,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="171">
   <si>
     <t>REPORT DATE:</t>
   </si>
@@ -598,6 +598,9 @@
   <si>
     <t xml:space="preserve">رقم العميل
 </t>
+  </si>
+  <si>
+    <t>Safaa Karim</t>
   </si>
 </sst>
 </file>
@@ -18196,7 +18199,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:O322"/>
+  <dimension ref="A1:O323"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="50.83203125" defaultRowHeight="50" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="42.83203125" style="1" customWidth="1"/>
@@ -18597,7 +18600,7 @@
     <row r="20" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="65"/>
       <c r="B20" s="43" t="s">
-        <v>65</v>
+        <v>170</v>
       </c>
       <c r="C20" s="24">
         <f ca="1">IFERROR(
@@ -18620,7 +18623,7 @@
     <row r="21" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="65"/>
       <c r="B21" s="43" t="s">
-        <v>155</v>
+        <v>65</v>
       </c>
       <c r="C21" s="24">
         <f ca="1">IFERROR(
@@ -18643,7 +18646,7 @@
     <row r="22" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="65"/>
       <c r="B22" s="43" t="s">
-        <v>31</v>
+        <v>155</v>
       </c>
       <c r="C22" s="24">
         <f ca="1">IFERROR(
@@ -18666,7 +18669,7 @@
     <row r="23" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="65"/>
       <c r="B23" s="43" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="C23" s="24">
         <f ca="1">IFERROR(
@@ -18686,19 +18689,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:4" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="63"/>
-      <c r="B24" s="27" t="s">
-        <v>58</v>
-      </c>
-      <c r="C24" s="26">
+    <row r="24" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="65"/>
+      <c r="B24" s="43" t="s">
+        <v>21</v>
+      </c>
+      <c r="C24" s="24">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A24) &amp; "'!C:C"), B24),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D24" s="87" cm="1">
+      <c r="D24" s="73" cm="1">
         <f t="array" aca="1" ref="D24" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A24&lt;&gt;""),$A$7:A24) &amp; "'!C:C"), $B24,
@@ -18710,20 +18713,18 @@
       </c>
     </row>
     <row r="25" spans="1:4" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="57" t="s">
-        <v>56</v>
-      </c>
-      <c r="B25" s="29" t="s">
-        <v>74</v>
-      </c>
-      <c r="C25" s="24">
+      <c r="A25" s="63"/>
+      <c r="B25" s="27" t="s">
+        <v>58</v>
+      </c>
+      <c r="C25" s="26">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A25) &amp; "'!C:C"), B25),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D25" s="88" cm="1">
+      <c r="D25" s="87" cm="1">
         <f t="array" aca="1" ref="D25" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A25&lt;&gt;""),$A$7:A25) &amp; "'!C:C"), $B25,
@@ -18735,9 +18736,11 @@
       </c>
     </row>
     <row r="26" spans="1:4" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="28"/>
+      <c r="A26" s="57" t="s">
+        <v>56</v>
+      </c>
       <c r="B26" s="29" t="s">
-        <v>59</v>
+        <v>74</v>
       </c>
       <c r="C26" s="24">
         <f ca="1">IFERROR(
@@ -18746,7 +18749,7 @@
 )</f>
         <v>0</v>
       </c>
-      <c r="D26" s="73" cm="1">
+      <c r="D26" s="88" cm="1">
         <f t="array" aca="1" ref="D26" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A26&lt;&gt;""),$A$7:A26) &amp; "'!C:C"), $B26,
@@ -18760,7 +18763,7 @@
     <row r="27" spans="1:4" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="28"/>
       <c r="B27" s="29" t="s">
-        <v>41</v>
+        <v>59</v>
       </c>
       <c r="C27" s="24">
         <f ca="1">IFERROR(
@@ -18783,7 +18786,7 @@
     <row r="28" spans="1:4" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="28"/>
       <c r="B28" s="29" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="C28" s="24">
         <f ca="1">IFERROR(
@@ -18806,7 +18809,7 @@
     <row r="29" spans="1:4" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="28"/>
       <c r="B29" s="29" t="s">
-        <v>81</v>
+        <v>36</v>
       </c>
       <c r="C29" s="24">
         <f ca="1">IFERROR(
@@ -18827,9 +18830,9 @@
       </c>
     </row>
     <row r="30" spans="1:4" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="38"/>
-      <c r="B30" s="43" t="s">
-        <v>158</v>
+      <c r="A30" s="28"/>
+      <c r="B30" s="29" t="s">
+        <v>81</v>
       </c>
       <c r="C30" s="24">
         <f ca="1">IFERROR(
@@ -18852,7 +18855,7 @@
     <row r="31" spans="1:4" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="38"/>
       <c r="B31" s="43" t="s">
-        <v>84</v>
+        <v>158</v>
       </c>
       <c r="C31" s="24">
         <f ca="1">IFERROR(
@@ -18875,16 +18878,16 @@
     <row r="32" spans="1:4" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="38"/>
       <c r="B32" s="43" t="s">
-        <v>43</v>
-      </c>
-      <c r="C32" s="26">
+        <v>84</v>
+      </c>
+      <c r="C32" s="24">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A32) &amp; "'!C:C"), B32),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D32" s="87" cm="1">
+      <c r="D32" s="73" cm="1">
         <f t="array" aca="1" ref="D32" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A32&lt;&gt;""),$A$7:A32) &amp; "'!C:C"), $B32,
@@ -18896,20 +18899,18 @@
       </c>
     </row>
     <row r="33" spans="1:4" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="69" t="s">
-        <v>44</v>
-      </c>
-      <c r="B33" s="46" t="s">
-        <v>75</v>
-      </c>
-      <c r="C33" s="47">
+      <c r="A33" s="38"/>
+      <c r="B33" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="C33" s="26">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A33) &amp; "'!C:C"), B33),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D33" s="88" cm="1">
+      <c r="D33" s="87" cm="1">
         <f t="array" aca="1" ref="D33" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A33&lt;&gt;""),$A$7:A33) &amp; "'!C:C"), $B33,
@@ -18921,18 +18922,20 @@
       </c>
     </row>
     <row r="34" spans="1:4" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="70"/>
-      <c r="B34" s="25" t="s">
-        <v>76</v>
-      </c>
-      <c r="C34" s="28">
+      <c r="A34" s="69" t="s">
+        <v>44</v>
+      </c>
+      <c r="B34" s="46" t="s">
+        <v>75</v>
+      </c>
+      <c r="C34" s="47">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A34) &amp; "'!C:C"), B34),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D34" s="73" cm="1">
+      <c r="D34" s="88" cm="1">
         <f t="array" aca="1" ref="D34" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A34&lt;&gt;""),$A$7:A34) &amp; "'!C:C"), $B34,
@@ -18946,7 +18949,7 @@
     <row r="35" spans="1:4" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="70"/>
       <c r="B35" s="25" t="s">
-        <v>165</v>
+        <v>76</v>
       </c>
       <c r="C35" s="28">
         <f ca="1">IFERROR(
@@ -18969,7 +18972,7 @@
     <row r="36" spans="1:4" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="70"/>
       <c r="B36" s="25" t="s">
-        <v>16</v>
+        <v>165</v>
       </c>
       <c r="C36" s="28">
         <f ca="1">IFERROR(
@@ -18990,9 +18993,9 @@
       </c>
     </row>
     <row r="37" spans="1:4" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="28"/>
-      <c r="B37" s="29" t="s">
-        <v>35</v>
+      <c r="A37" s="70"/>
+      <c r="B37" s="25" t="s">
+        <v>16</v>
       </c>
       <c r="C37" s="28">
         <f ca="1">IFERROR(
@@ -19015,7 +19018,7 @@
     <row r="38" spans="1:4" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="28"/>
       <c r="B38" s="29" t="s">
-        <v>77</v>
+        <v>35</v>
       </c>
       <c r="C38" s="28">
         <f ca="1">IFERROR(
@@ -19038,7 +19041,7 @@
     <row r="39" spans="1:4" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="28"/>
       <c r="B39" s="29" t="s">
-        <v>37</v>
+        <v>77</v>
       </c>
       <c r="C39" s="28">
         <f ca="1">IFERROR(
@@ -19059,18 +19062,18 @@
       </c>
     </row>
     <row r="40" spans="1:4" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="80"/>
-      <c r="B40" s="75" t="s">
-        <v>15</v>
-      </c>
-      <c r="C40" s="26">
+      <c r="A40" s="28"/>
+      <c r="B40" s="29" t="s">
+        <v>37</v>
+      </c>
+      <c r="C40" s="28">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A40) &amp; "'!C:C"), B40),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D40" s="87" cm="1">
+      <c r="D40" s="73" cm="1">
         <f t="array" aca="1" ref="D40" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A40&lt;&gt;""),$A$7:A40) &amp; "'!C:C"), $B40,
@@ -19082,20 +19085,18 @@
       </c>
     </row>
     <row r="41" spans="1:4" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="84" t="s">
-        <v>93</v>
-      </c>
-      <c r="B41" s="83" t="s">
-        <v>138</v>
-      </c>
-      <c r="C41" s="82">
+      <c r="A41" s="80"/>
+      <c r="B41" s="75" t="s">
+        <v>15</v>
+      </c>
+      <c r="C41" s="26">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A41) &amp; "'!C:C"), B41),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D41" s="88" cm="1">
+      <c r="D41" s="87" cm="1">
         <f t="array" aca="1" ref="D41" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A41&lt;&gt;""),$A$7:A41) &amp; "'!C:C"), $B41,
@@ -19107,18 +19108,20 @@
       </c>
     </row>
     <row r="42" spans="1:4" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="31"/>
-      <c r="B42" s="29" t="s">
-        <v>137</v>
-      </c>
-      <c r="C42" s="28">
+      <c r="A42" s="84" t="s">
+        <v>93</v>
+      </c>
+      <c r="B42" s="83" t="s">
+        <v>138</v>
+      </c>
+      <c r="C42" s="82">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A42) &amp; "'!C:C"), B42),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D42" s="73" cm="1">
+      <c r="D42" s="88" cm="1">
         <f t="array" aca="1" ref="D42" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A42&lt;&gt;""),$A$7:A42) &amp; "'!C:C"), $B42,
@@ -19130,9 +19133,9 @@
       </c>
     </row>
     <row r="43" spans="1:4" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="73"/>
+      <c r="A43" s="31"/>
       <c r="B43" s="29" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C43" s="28">
         <f ca="1">IFERROR(
@@ -19152,10 +19155,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:4" s="14" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="28"/>
+    <row r="44" spans="1:4" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A44" s="73"/>
       <c r="B44" s="29" t="s">
-        <v>63</v>
+        <v>136</v>
       </c>
       <c r="C44" s="28">
         <f ca="1">IFERROR(
@@ -19175,10 +19178,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:4" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:4" s="14" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="28"/>
       <c r="B45" s="29" t="s">
-        <v>135</v>
+        <v>63</v>
       </c>
       <c r="C45" s="28">
         <f ca="1">IFERROR(
@@ -19201,7 +19204,7 @@
     <row r="46" spans="1:4" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="28"/>
       <c r="B46" s="29" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C46" s="28">
         <f ca="1">IFERROR(
@@ -19222,18 +19225,18 @@
       </c>
     </row>
     <row r="47" spans="1:4" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="80"/>
-      <c r="B47" s="75" t="s">
-        <v>133</v>
-      </c>
-      <c r="C47" s="80">
+      <c r="A47" s="28"/>
+      <c r="B47" s="29" t="s">
+        <v>134</v>
+      </c>
+      <c r="C47" s="28">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A47) &amp; "'!C:C"), B47),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D47" s="87" cm="1">
+      <c r="D47" s="73" cm="1">
         <f t="array" aca="1" ref="D47" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A47&lt;&gt;""),$A$7:A47) &amp; "'!C:C"), $B47,
@@ -19245,20 +19248,18 @@
       </c>
     </row>
     <row r="48" spans="1:4" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="57" t="s">
-        <v>92</v>
-      </c>
-      <c r="B48" s="29" t="s">
-        <v>132</v>
-      </c>
-      <c r="C48" s="28">
+      <c r="A48" s="80"/>
+      <c r="B48" s="75" t="s">
+        <v>133</v>
+      </c>
+      <c r="C48" s="80">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A48) &amp; "'!C:C"), B48),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D48" s="88" cm="1">
+      <c r="D48" s="87" cm="1">
         <f t="array" aca="1" ref="D48" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A48&lt;&gt;""),$A$7:A48) &amp; "'!C:C"), $B48,
@@ -19270,9 +19271,11 @@
       </c>
     </row>
     <row r="49" spans="1:4" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="57"/>
+      <c r="A49" s="57" t="s">
+        <v>92</v>
+      </c>
       <c r="B49" s="29" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C49" s="28">
         <f ca="1">IFERROR(
@@ -19281,7 +19284,7 @@
 )</f>
         <v>0</v>
       </c>
-      <c r="D49" s="73" cm="1">
+      <c r="D49" s="88" cm="1">
         <f t="array" aca="1" ref="D49" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A49&lt;&gt;""),$A$7:A49) &amp; "'!C:C"), $B49,
@@ -19295,7 +19298,7 @@
     <row r="50" spans="1:4" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="57"/>
       <c r="B50" s="29" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C50" s="28">
         <f ca="1">IFERROR(
@@ -19316,9 +19319,9 @@
       </c>
     </row>
     <row r="51" spans="1:4" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="31"/>
+      <c r="A51" s="57"/>
       <c r="B51" s="29" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C51" s="28">
         <f ca="1">IFERROR(
@@ -19341,7 +19344,7 @@
     <row r="52" spans="1:4" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="31"/>
       <c r="B52" s="29" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C52" s="28">
         <f ca="1">IFERROR(
@@ -19362,9 +19365,9 @@
       </c>
     </row>
     <row r="53" spans="1:4" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="65"/>
-      <c r="B53" s="43" t="s">
-        <v>127</v>
+      <c r="A53" s="31"/>
+      <c r="B53" s="29" t="s">
+        <v>128</v>
       </c>
       <c r="C53" s="28">
         <f ca="1">IFERROR(
@@ -19385,18 +19388,18 @@
       </c>
     </row>
     <row r="54" spans="1:4" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="81"/>
-      <c r="B54" s="75" t="s">
-        <v>126</v>
-      </c>
-      <c r="C54" s="80">
+      <c r="A54" s="65"/>
+      <c r="B54" s="43" t="s">
+        <v>127</v>
+      </c>
+      <c r="C54" s="28">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A54) &amp; "'!C:C"), B54),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D54" s="87" cm="1">
+      <c r="D54" s="73" cm="1">
         <f t="array" aca="1" ref="D54" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A54&lt;&gt;""),$A$7:A54) &amp; "'!C:C"), $B54,
@@ -19408,20 +19411,18 @@
       </c>
     </row>
     <row r="55" spans="1:4" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="57" t="s">
-        <v>91</v>
-      </c>
-      <c r="B55" s="29" t="s">
-        <v>125</v>
-      </c>
-      <c r="C55" s="28">
+      <c r="A55" s="81"/>
+      <c r="B55" s="75" t="s">
+        <v>126</v>
+      </c>
+      <c r="C55" s="80">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A55) &amp; "'!C:C"), B55),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D55" s="88" cm="1">
+      <c r="D55" s="87" cm="1">
         <f t="array" aca="1" ref="D55" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A55&lt;&gt;""),$A$7:A55) &amp; "'!C:C"), $B55,
@@ -19433,9 +19434,11 @@
       </c>
     </row>
     <row r="56" spans="1:4" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A56" s="62"/>
+      <c r="A56" s="57" t="s">
+        <v>91</v>
+      </c>
       <c r="B56" s="29" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C56" s="28">
         <f ca="1">IFERROR(
@@ -19444,7 +19447,7 @@
 )</f>
         <v>0</v>
       </c>
-      <c r="D56" s="73" cm="1">
+      <c r="D56" s="88" cm="1">
         <f t="array" aca="1" ref="D56" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A56&lt;&gt;""),$A$7:A56) &amp; "'!C:C"), $B56,
@@ -19458,7 +19461,7 @@
     <row r="57" spans="1:4" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="62"/>
       <c r="B57" s="29" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C57" s="28">
         <f ca="1">IFERROR(
@@ -19481,7 +19484,7 @@
     <row r="58" spans="1:4" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="62"/>
       <c r="B58" s="29" t="s">
-        <v>157</v>
+        <v>123</v>
       </c>
       <c r="C58" s="28">
         <f ca="1">IFERROR(
@@ -19502,9 +19505,9 @@
       </c>
     </row>
     <row r="59" spans="1:4" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A59" s="28"/>
+      <c r="A59" s="62"/>
       <c r="B59" s="29" t="s">
-        <v>121</v>
+        <v>157</v>
       </c>
       <c r="C59" s="28">
         <f ca="1">IFERROR(
@@ -19525,18 +19528,18 @@
       </c>
     </row>
     <row r="60" spans="1:4" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A60" s="26"/>
-      <c r="B60" s="27" t="s">
-        <v>120</v>
-      </c>
-      <c r="C60" s="26">
+      <c r="A60" s="28"/>
+      <c r="B60" s="29" t="s">
+        <v>121</v>
+      </c>
+      <c r="C60" s="28">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A60) &amp; "'!C:C"), B60),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D60" s="87" cm="1">
+      <c r="D60" s="73" cm="1">
         <f t="array" aca="1" ref="D60" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A60&lt;&gt;""),$A$7:A60) &amp; "'!C:C"), $B60,
@@ -19548,20 +19551,18 @@
       </c>
     </row>
     <row r="61" spans="1:4" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A61" s="71" t="s">
-        <v>53</v>
-      </c>
-      <c r="B61" s="46" t="s">
-        <v>13</v>
-      </c>
-      <c r="C61" s="47">
+      <c r="A61" s="26"/>
+      <c r="B61" s="27" t="s">
+        <v>120</v>
+      </c>
+      <c r="C61" s="26">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A61) &amp; "'!C:C"), B61),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D61" s="88" cm="1">
+      <c r="D61" s="87" cm="1">
         <f t="array" aca="1" ref="D61" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A61&lt;&gt;""),$A$7:A61) &amp; "'!C:C"), $B61,
@@ -19573,18 +19574,20 @@
       </c>
     </row>
     <row r="62" spans="1:4" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A62" s="62"/>
-      <c r="B62" s="29" t="s">
-        <v>66</v>
-      </c>
-      <c r="C62" s="28">
+      <c r="A62" s="71" t="s">
+        <v>53</v>
+      </c>
+      <c r="B62" s="46" t="s">
+        <v>13</v>
+      </c>
+      <c r="C62" s="47">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A62) &amp; "'!C:C"), B62),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D62" s="73" cm="1">
+      <c r="D62" s="88" cm="1">
         <f t="array" aca="1" ref="D62" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A62&lt;&gt;""),$A$7:A62) &amp; "'!C:C"), $B62,
@@ -19598,7 +19601,7 @@
     <row r="63" spans="1:4" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="62"/>
       <c r="B63" s="29" t="s">
-        <v>156</v>
+        <v>66</v>
       </c>
       <c r="C63" s="28">
         <f ca="1">IFERROR(
@@ -19621,7 +19624,7 @@
     <row r="64" spans="1:4" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="62"/>
       <c r="B64" s="29" t="s">
-        <v>32</v>
+        <v>156</v>
       </c>
       <c r="C64" s="28">
         <f ca="1">IFERROR(
@@ -19644,7 +19647,7 @@
     <row r="65" spans="1:15" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="62"/>
       <c r="B65" s="29" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C65" s="28">
         <f ca="1">IFERROR(
@@ -19665,9 +19668,9 @@
       </c>
     </row>
     <row r="66" spans="1:15" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A66" s="28"/>
+      <c r="A66" s="62"/>
       <c r="B66" s="29" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C66" s="28">
         <f ca="1">IFERROR(
@@ -19688,9 +19691,9 @@
       </c>
     </row>
     <row r="67" spans="1:15" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A67" s="38"/>
-      <c r="B67" s="43" t="s">
-        <v>82</v>
+      <c r="A67" s="28"/>
+      <c r="B67" s="29" t="s">
+        <v>34</v>
       </c>
       <c r="C67" s="28">
         <f ca="1">IFERROR(
@@ -19711,9 +19714,9 @@
       </c>
     </row>
     <row r="68" spans="1:15" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A68" s="28"/>
-      <c r="B68" s="29" t="s">
-        <v>11</v>
+      <c r="A68" s="38"/>
+      <c r="B68" s="43" t="s">
+        <v>82</v>
       </c>
       <c r="C68" s="28">
         <f ca="1">IFERROR(
@@ -19722,7 +19725,7 @@
 )</f>
         <v>0</v>
       </c>
-      <c r="D68" s="87" cm="1">
+      <c r="D68" s="73" cm="1">
         <f t="array" aca="1" ref="D68" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A68&lt;&gt;""),$A$7:A68) &amp; "'!C:C"), $B68,
@@ -19734,11 +19737,11 @@
       </c>
     </row>
     <row r="69" spans="1:15" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A69" s="90"/>
-      <c r="B69" s="91" t="s">
-        <v>18</v>
-      </c>
-      <c r="C69" s="90">
+      <c r="A69" s="28"/>
+      <c r="B69" s="29" t="s">
+        <v>11</v>
+      </c>
+      <c r="C69" s="28">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A69) &amp; "'!C:C"), B69),
    0
@@ -19755,33 +19758,20 @@
 0)</f>
         <v>0</v>
       </c>
-      <c r="E69" s="1"/>
-      <c r="F69" s="1"/>
-      <c r="G69" s="1"/>
-      <c r="H69" s="1"/>
-      <c r="I69" s="1"/>
-      <c r="J69" s="1"/>
-      <c r="K69" s="1"/>
-      <c r="L69" s="1"/>
-      <c r="M69" s="1"/>
-      <c r="N69" s="1"/>
-      <c r="O69" s="1"/>
     </row>
     <row r="70" spans="1:15" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A70" s="71" t="s">
-        <v>54</v>
-      </c>
-      <c r="B70" s="46" t="s">
-        <v>23</v>
-      </c>
-      <c r="C70" s="47">
+      <c r="A70" s="90"/>
+      <c r="B70" s="91" t="s">
+        <v>18</v>
+      </c>
+      <c r="C70" s="90">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A70) &amp; "'!C:C"), B70),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D70" s="88" cm="1">
+      <c r="D70" s="87" cm="1">
         <f t="array" aca="1" ref="D70" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A70&lt;&gt;""),$A$7:A70) &amp; "'!C:C"), $B70,
@@ -19791,20 +19781,33 @@
 0)</f>
         <v>0</v>
       </c>
+      <c r="E70" s="1"/>
+      <c r="F70" s="1"/>
+      <c r="G70" s="1"/>
+      <c r="H70" s="1"/>
+      <c r="I70" s="1"/>
+      <c r="J70" s="1"/>
+      <c r="K70" s="1"/>
+      <c r="L70" s="1"/>
+      <c r="M70" s="1"/>
+      <c r="N70" s="1"/>
+      <c r="O70" s="1"/>
     </row>
     <row r="71" spans="1:15" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A71" s="28"/>
-      <c r="B71" s="29" t="s">
-        <v>24</v>
-      </c>
-      <c r="C71" s="28">
+      <c r="A71" s="71" t="s">
+        <v>54</v>
+      </c>
+      <c r="B71" s="46" t="s">
+        <v>23</v>
+      </c>
+      <c r="C71" s="47">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A71) &amp; "'!C:C"), B71),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D71" s="73" cm="1">
+      <c r="D71" s="88" cm="1">
         <f t="array" aca="1" ref="D71" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A71&lt;&gt;""),$A$7:A71) &amp; "'!C:C"), $B71,
@@ -19818,7 +19821,7 @@
     <row r="72" spans="1:15" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="28"/>
       <c r="B72" s="29" t="s">
-        <v>163</v>
+        <v>24</v>
       </c>
       <c r="C72" s="28">
         <f ca="1">IFERROR(
@@ -19841,7 +19844,7 @@
     <row r="73" spans="1:15" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="28"/>
       <c r="B73" s="29" t="s">
-        <v>17</v>
+        <v>163</v>
       </c>
       <c r="C73" s="28">
         <f ca="1">IFERROR(
@@ -19864,7 +19867,7 @@
     <row r="74" spans="1:15" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="28"/>
       <c r="B74" s="29" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="C74" s="28">
         <f ca="1">IFERROR(
@@ -19886,8 +19889,8 @@
     </row>
     <row r="75" spans="1:15" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="28"/>
-      <c r="B75" s="92" t="s">
-        <v>161</v>
+      <c r="B75" s="29" t="s">
+        <v>12</v>
       </c>
       <c r="C75" s="28">
         <f ca="1">IFERROR(
@@ -19907,10 +19910,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:15" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:15" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="28"/>
-      <c r="B76" s="29" t="s">
-        <v>73</v>
+      <c r="B76" s="92" t="s">
+        <v>161</v>
       </c>
       <c r="C76" s="28">
         <f ca="1">IFERROR(
@@ -19919,7 +19922,7 @@
 )</f>
         <v>0</v>
       </c>
-      <c r="D76" s="87" cm="1">
+      <c r="D76" s="73" cm="1">
         <f t="array" aca="1" ref="D76" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A76&lt;&gt;""),$A$7:A76) &amp; "'!C:C"), $B76,
@@ -19930,19 +19933,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:15" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A77" s="24"/>
-      <c r="B77" s="25" t="s">
-        <v>39</v>
-      </c>
-      <c r="C77" s="24">
+    <row r="77" spans="1:15" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A77" s="28"/>
+      <c r="B77" s="29" t="s">
+        <v>73</v>
+      </c>
+      <c r="C77" s="28">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A77) &amp; "'!C:C"), B77),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D77" s="73" cm="1">
+      <c r="D77" s="87" cm="1">
         <f t="array" aca="1" ref="D77" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A77&lt;&gt;""),$A$7:A77) &amp; "'!C:C"), $B77,
@@ -19954,20 +19957,18 @@
       </c>
     </row>
     <row r="78" spans="1:15" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A78" s="72" t="s">
-        <v>55</v>
-      </c>
-      <c r="B78" s="44" t="s">
-        <v>68</v>
-      </c>
-      <c r="C78" s="45">
+      <c r="A78" s="24"/>
+      <c r="B78" s="25" t="s">
+        <v>39</v>
+      </c>
+      <c r="C78" s="24">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A78) &amp; "'!C:C"), B78),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D78" s="88" cm="1">
+      <c r="D78" s="73" cm="1">
         <f t="array" aca="1" ref="D78" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A78&lt;&gt;""),$A$7:A78) &amp; "'!C:C"), $B78,
@@ -19977,31 +19978,22 @@
 0)</f>
         <v>0</v>
       </c>
-      <c r="E78" s="1"/>
-      <c r="F78" s="1"/>
-      <c r="G78" s="1"/>
-      <c r="H78" s="1"/>
-      <c r="I78" s="1"/>
-      <c r="J78" s="1"/>
-      <c r="K78" s="1"/>
-      <c r="L78" s="1"/>
-      <c r="M78" s="1"/>
-      <c r="N78" s="1"/>
-      <c r="O78" s="1"/>
     </row>
     <row r="79" spans="1:15" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A79" s="28"/>
-      <c r="B79" s="29" t="s">
-        <v>69</v>
-      </c>
-      <c r="C79" s="28">
+      <c r="A79" s="72" t="s">
+        <v>55</v>
+      </c>
+      <c r="B79" s="44" t="s">
+        <v>68</v>
+      </c>
+      <c r="C79" s="45">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A79) &amp; "'!C:C"), B79),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D79" s="73" cm="1">
+      <c r="D79" s="88" cm="1">
         <f t="array" aca="1" ref="D79" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A79&lt;&gt;""),$A$7:A79) &amp; "'!C:C"), $B79,
@@ -20026,7 +20018,7 @@
     <row r="80" spans="1:15" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" s="28"/>
       <c r="B80" s="29" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C80" s="28">
         <f ca="1">IFERROR(
@@ -20060,7 +20052,7 @@
     <row r="81" spans="1:15" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="28"/>
       <c r="B81" s="29" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C81" s="28">
         <f ca="1">IFERROR(
@@ -20079,11 +20071,22 @@
 0)</f>
         <v>0</v>
       </c>
+      <c r="E81" s="1"/>
+      <c r="F81" s="1"/>
+      <c r="G81" s="1"/>
+      <c r="H81" s="1"/>
+      <c r="I81" s="1"/>
+      <c r="J81" s="1"/>
+      <c r="K81" s="1"/>
+      <c r="L81" s="1"/>
+      <c r="M81" s="1"/>
+      <c r="N81" s="1"/>
+      <c r="O81" s="1"/>
     </row>
     <row r="82" spans="1:15" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" s="28"/>
       <c r="B82" s="29" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C82" s="28">
         <f ca="1">IFERROR(
@@ -20102,22 +20105,11 @@
 0)</f>
         <v>0</v>
       </c>
-      <c r="E82" s="1"/>
-      <c r="F82" s="1"/>
-      <c r="G82" s="1"/>
-      <c r="H82" s="1"/>
-      <c r="I82" s="1"/>
-      <c r="J82" s="1"/>
-      <c r="K82" s="1"/>
-      <c r="L82" s="1"/>
-      <c r="M82" s="1"/>
-      <c r="N82" s="1"/>
-      <c r="O82" s="1"/>
     </row>
     <row r="83" spans="1:15" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="28"/>
       <c r="B83" s="29" t="s">
-        <v>30</v>
+        <v>71</v>
       </c>
       <c r="C83" s="28">
         <f ca="1">IFERROR(
@@ -20151,7 +20143,7 @@
     <row r="84" spans="1:15" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" s="28"/>
       <c r="B84" s="29" t="s">
-        <v>72</v>
+        <v>30</v>
       </c>
       <c r="C84" s="28">
         <f ca="1">IFERROR(
@@ -20182,10 +20174,10 @@
       <c r="N84" s="1"/>
       <c r="O84" s="1"/>
     </row>
-    <row r="85" spans="1:15" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:15" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A85" s="28"/>
       <c r="B85" s="29" t="s">
-        <v>40</v>
+        <v>72</v>
       </c>
       <c r="C85" s="28">
         <f ca="1">IFERROR(
@@ -20204,22 +20196,31 @@
 0)</f>
         <v>0</v>
       </c>
+      <c r="E85" s="1"/>
+      <c r="F85" s="1"/>
+      <c r="G85" s="1"/>
+      <c r="H85" s="1"/>
+      <c r="I85" s="1"/>
+      <c r="J85" s="1"/>
+      <c r="K85" s="1"/>
+      <c r="L85" s="1"/>
+      <c r="M85" s="1"/>
+      <c r="N85" s="1"/>
+      <c r="O85" s="1"/>
     </row>
     <row r="86" spans="1:15" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A86" s="69" t="s">
-        <v>57</v>
-      </c>
-      <c r="B86" s="48" t="s">
-        <v>27</v>
-      </c>
-      <c r="C86" s="47">
+      <c r="A86" s="28"/>
+      <c r="B86" s="29" t="s">
+        <v>40</v>
+      </c>
+      <c r="C86" s="28">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A86) &amp; "'!C:C"), B86),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D86" s="88" cm="1">
+      <c r="D86" s="73" cm="1">
         <f t="array" aca="1" ref="D86" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A86&lt;&gt;""),$A$7:A86) &amp; "'!C:C"), $B86,
@@ -20231,18 +20232,20 @@
       </c>
     </row>
     <row r="87" spans="1:15" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A87" s="31"/>
-      <c r="B87" s="30" t="s">
-        <v>78</v>
-      </c>
-      <c r="C87" s="28">
+      <c r="A87" s="69" t="s">
+        <v>57</v>
+      </c>
+      <c r="B87" s="48" t="s">
+        <v>27</v>
+      </c>
+      <c r="C87" s="47">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A87) &amp; "'!C:C"), B87),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D87" s="73" cm="1">
+      <c r="D87" s="88" cm="1">
         <f t="array" aca="1" ref="D87" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A87&lt;&gt;""),$A$7:A87) &amp; "'!C:C"), $B87,
@@ -20256,7 +20259,7 @@
     <row r="88" spans="1:15" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" s="31"/>
       <c r="B88" s="30" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C88" s="28">
         <f ca="1">IFERROR(
@@ -20279,7 +20282,7 @@
     <row r="89" spans="1:15" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A89" s="31"/>
       <c r="B89" s="30" t="s">
-        <v>28</v>
+        <v>79</v>
       </c>
       <c r="C89" s="28">
         <f ca="1">IFERROR(
@@ -20302,7 +20305,7 @@
     <row r="90" spans="1:15" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A90" s="31"/>
       <c r="B90" s="30" t="s">
-        <v>164</v>
+        <v>28</v>
       </c>
       <c r="C90" s="28">
         <f ca="1">IFERROR(
@@ -20325,7 +20328,7 @@
     <row r="91" spans="1:15" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91" s="31"/>
       <c r="B91" s="30" t="s">
-        <v>29</v>
+        <v>164</v>
       </c>
       <c r="C91" s="28">
         <f ca="1">IFERROR(
@@ -20348,7 +20351,7 @@
     <row r="92" spans="1:15" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A92" s="31"/>
       <c r="B92" s="30" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="C92" s="28">
         <f ca="1">IFERROR(
@@ -20369,9 +20372,9 @@
       </c>
     </row>
     <row r="93" spans="1:15" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A93" s="65"/>
-      <c r="B93" s="66" t="s">
-        <v>83</v>
+      <c r="A93" s="31"/>
+      <c r="B93" s="30" t="s">
+        <v>38</v>
       </c>
       <c r="C93" s="28">
         <f ca="1">IFERROR(
@@ -20392,18 +20395,18 @@
       </c>
     </row>
     <row r="94" spans="1:15" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A94" s="81"/>
-      <c r="B94" s="85" t="s">
-        <v>80</v>
-      </c>
-      <c r="C94" s="80">
+      <c r="A94" s="65"/>
+      <c r="B94" s="66" t="s">
+        <v>83</v>
+      </c>
+      <c r="C94" s="28">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A94) &amp; "'!C:C"), B94),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D94" s="87" cm="1">
+      <c r="D94" s="73" cm="1">
         <f t="array" aca="1" ref="D94" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A94&lt;&gt;""),$A$7:A94) &amp; "'!C:C"), $B94,
@@ -20415,20 +20418,18 @@
       </c>
     </row>
     <row r="95" spans="1:15" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A95" s="24" t="s">
-        <v>88</v>
-      </c>
-      <c r="B95" s="29" t="s">
-        <v>104</v>
-      </c>
-      <c r="C95" s="24">
+      <c r="A95" s="81"/>
+      <c r="B95" s="85" t="s">
+        <v>80</v>
+      </c>
+      <c r="C95" s="80">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A95) &amp; "'!C:C"), B95),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D95" s="88" cm="1">
+      <c r="D95" s="87" cm="1">
         <f t="array" aca="1" ref="D95" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A95&lt;&gt;""),$A$7:A95) &amp; "'!C:C"), $B95,
@@ -20440,18 +20441,20 @@
       </c>
     </row>
     <row r="96" spans="1:15" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A96" s="73"/>
+      <c r="A96" s="24" t="s">
+        <v>88</v>
+      </c>
       <c r="B96" s="29" t="s">
-        <v>103</v>
-      </c>
-      <c r="C96" s="28">
+        <v>104</v>
+      </c>
+      <c r="C96" s="24">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A96) &amp; "'!C:C"), B96),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D96" s="73" cm="1">
+      <c r="D96" s="88" cm="1">
         <f t="array" aca="1" ref="D96" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A96&lt;&gt;""),$A$7:A96) &amp; "'!C:C"), $B96,
@@ -20463,9 +20466,9 @@
       </c>
     </row>
     <row r="97" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A97" s="28"/>
+      <c r="A97" s="73"/>
       <c r="B97" s="29" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C97" s="28">
         <f ca="1">IFERROR(
@@ -20488,7 +20491,7 @@
     <row r="98" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98" s="28"/>
       <c r="B98" s="29" t="s">
-        <v>159</v>
+        <v>102</v>
       </c>
       <c r="C98" s="28">
         <f ca="1">IFERROR(
@@ -20511,7 +20514,7 @@
     <row r="99" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A99" s="28"/>
       <c r="B99" s="29" t="s">
-        <v>101</v>
+        <v>159</v>
       </c>
       <c r="C99" s="28">
         <f ca="1">IFERROR(
@@ -20532,18 +20535,18 @@
       </c>
     </row>
     <row r="100" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A100" s="80"/>
-      <c r="B100" s="75" t="s">
-        <v>100</v>
-      </c>
-      <c r="C100" s="80">
+      <c r="A100" s="28"/>
+      <c r="B100" s="29" t="s">
+        <v>101</v>
+      </c>
+      <c r="C100" s="28">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A100) &amp; "'!C:C"), B100),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D100" s="87" cm="1">
+      <c r="D100" s="73" cm="1">
         <f t="array" aca="1" ref="D100" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A100&lt;&gt;""),$A$7:A100) &amp; "'!C:C"), $B100,
@@ -20555,20 +20558,18 @@
       </c>
     </row>
     <row r="101" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A101" s="24" t="s">
-        <v>90</v>
-      </c>
-      <c r="B101" s="25" t="s">
-        <v>119</v>
-      </c>
-      <c r="C101" s="24">
+      <c r="A101" s="80"/>
+      <c r="B101" s="75" t="s">
+        <v>100</v>
+      </c>
+      <c r="C101" s="80">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A101) &amp; "'!C:C"), B101),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D101" s="88" cm="1">
+      <c r="D101" s="87" cm="1">
         <f t="array" aca="1" ref="D101" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A101&lt;&gt;""),$A$7:A101) &amp; "'!C:C"), $B101,
@@ -20580,18 +20581,20 @@
       </c>
     </row>
     <row r="102" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A102" s="28"/>
-      <c r="B102" s="29" t="s">
-        <v>118</v>
-      </c>
-      <c r="C102" s="28">
+      <c r="A102" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="B102" s="25" t="s">
+        <v>119</v>
+      </c>
+      <c r="C102" s="24">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A102) &amp; "'!C:C"), B102),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D102" s="73" cm="1">
+      <c r="D102" s="88" cm="1">
         <f t="array" aca="1" ref="D102" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A102&lt;&gt;""),$A$7:A102) &amp; "'!C:C"), $B102,
@@ -20605,7 +20608,7 @@
     <row r="103" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A103" s="28"/>
       <c r="B103" s="29" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C103" s="28">
         <f ca="1">IFERROR(
@@ -20628,7 +20631,7 @@
     <row r="104" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A104" s="28"/>
       <c r="B104" s="29" t="s">
-        <v>153</v>
+        <v>117</v>
       </c>
       <c r="C104" s="28">
         <f ca="1">IFERROR(
@@ -20651,7 +20654,7 @@
     <row r="105" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A105" s="28"/>
       <c r="B105" s="29" t="s">
-        <v>116</v>
+        <v>153</v>
       </c>
       <c r="C105" s="28">
         <f ca="1">IFERROR(
@@ -20674,7 +20677,7 @@
     <row r="106" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A106" s="28"/>
       <c r="B106" s="29" t="s">
-        <v>160</v>
+        <v>116</v>
       </c>
       <c r="C106" s="28">
         <f ca="1">IFERROR(
@@ -20697,7 +20700,7 @@
     <row r="107" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A107" s="28"/>
       <c r="B107" s="29" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="C107" s="28">
         <f ca="1">IFERROR(
@@ -20720,7 +20723,7 @@
     <row r="108" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A108" s="28"/>
       <c r="B108" s="29" t="s">
-        <v>115</v>
+        <v>167</v>
       </c>
       <c r="C108" s="28">
         <f ca="1">IFERROR(
@@ -20743,7 +20746,7 @@
     <row r="109" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A109" s="28"/>
       <c r="B109" s="29" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C109" s="28">
         <f ca="1">IFERROR(
@@ -20764,9 +20767,9 @@
       </c>
     </row>
     <row r="110" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A110" s="31"/>
-      <c r="B110" s="30" t="s">
-        <v>113</v>
+      <c r="A110" s="28"/>
+      <c r="B110" s="29" t="s">
+        <v>114</v>
       </c>
       <c r="C110" s="28">
         <f ca="1">IFERROR(
@@ -20789,7 +20792,7 @@
     <row r="111" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A111" s="31"/>
       <c r="B111" s="30" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C111" s="28">
         <f ca="1">IFERROR(
@@ -20810,18 +20813,18 @@
       </c>
     </row>
     <row r="112" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A112" s="79"/>
-      <c r="B112" s="78" t="s">
-        <v>111</v>
-      </c>
-      <c r="C112" s="77">
+      <c r="A112" s="31"/>
+      <c r="B112" s="30" t="s">
+        <v>112</v>
+      </c>
+      <c r="C112" s="28">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A112) &amp; "'!C:C"), B112),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D112" s="87" cm="1">
+      <c r="D112" s="73" cm="1">
         <f t="array" aca="1" ref="D112" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A112&lt;&gt;""),$A$7:A112) &amp; "'!C:C"), $B112,
@@ -20833,20 +20836,18 @@
       </c>
     </row>
     <row r="113" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A113" s="24" t="s">
-        <v>89</v>
-      </c>
-      <c r="B113" s="25" t="s">
-        <v>110</v>
-      </c>
-      <c r="C113" s="24">
+      <c r="A113" s="79"/>
+      <c r="B113" s="78" t="s">
+        <v>111</v>
+      </c>
+      <c r="C113" s="77">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A113) &amp; "'!C:C"), B113),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D113" s="88" cm="1">
+      <c r="D113" s="87" cm="1">
         <f t="array" aca="1" ref="D113" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A113&lt;&gt;""),$A$7:A113) &amp; "'!C:C"), $B113,
@@ -20858,18 +20859,20 @@
       </c>
     </row>
     <row r="114" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A114" s="28"/>
-      <c r="B114" s="29" t="s">
-        <v>109</v>
-      </c>
-      <c r="C114" s="28">
+      <c r="A114" s="24" t="s">
+        <v>89</v>
+      </c>
+      <c r="B114" s="25" t="s">
+        <v>110</v>
+      </c>
+      <c r="C114" s="24">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A114) &amp; "'!C:C"), B114),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D114" s="73" cm="1">
+      <c r="D114" s="88" cm="1">
         <f t="array" aca="1" ref="D114" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A114&lt;&gt;""),$A$7:A114) &amp; "'!C:C"), $B114,
@@ -20883,7 +20886,7 @@
     <row r="115" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A115" s="28"/>
       <c r="B115" s="29" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C115" s="28">
         <f ca="1">IFERROR(
@@ -20906,7 +20909,7 @@
     <row r="116" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A116" s="28"/>
       <c r="B116" s="29" t="s">
-        <v>162</v>
+        <v>108</v>
       </c>
       <c r="C116" s="28">
         <f ca="1">IFERROR(
@@ -20929,7 +20932,7 @@
     <row r="117" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A117" s="28"/>
       <c r="B117" s="29" t="s">
-        <v>107</v>
+        <v>162</v>
       </c>
       <c r="C117" s="28">
         <f ca="1">IFERROR(
@@ -20952,7 +20955,7 @@
     <row r="118" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A118" s="28"/>
       <c r="B118" s="29" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C118" s="28">
         <f ca="1">IFERROR(
@@ -20973,18 +20976,18 @@
       </c>
     </row>
     <row r="119" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A119" s="76"/>
-      <c r="B119" s="75" t="s">
-        <v>105</v>
-      </c>
-      <c r="C119" s="74">
+      <c r="A119" s="28"/>
+      <c r="B119" s="29" t="s">
+        <v>106</v>
+      </c>
+      <c r="C119" s="28">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A119) &amp; "'!C:C"), B119),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D119" s="87" cm="1">
+      <c r="D119" s="73" cm="1">
         <f t="array" aca="1" ref="D119" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A119&lt;&gt;""),$A$7:A119) &amp; "'!C:C"), $B119,
@@ -20996,20 +20999,18 @@
       </c>
     </row>
     <row r="120" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A120" s="69" t="s">
-        <v>87</v>
-      </c>
-      <c r="B120" s="66" t="s">
-        <v>99</v>
-      </c>
-      <c r="C120" s="47">
+      <c r="A120" s="76"/>
+      <c r="B120" s="75" t="s">
+        <v>105</v>
+      </c>
+      <c r="C120" s="74">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A120) &amp; "'!C:C"), B120),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D120" s="88" cm="1">
+      <c r="D120" s="87" cm="1">
         <f t="array" aca="1" ref="D120" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A120&lt;&gt;""),$A$7:A120) &amp; "'!C:C"), $B120,
@@ -21021,18 +21022,20 @@
       </c>
     </row>
     <row r="121" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A121" s="73"/>
-      <c r="B121" s="29" t="s">
-        <v>98</v>
-      </c>
-      <c r="C121" s="28">
+      <c r="A121" s="69" t="s">
+        <v>87</v>
+      </c>
+      <c r="B121" s="66" t="s">
+        <v>99</v>
+      </c>
+      <c r="C121" s="47">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A121) &amp; "'!C:C"), B121),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D121" s="73" cm="1">
+      <c r="D121" s="88" cm="1">
         <f t="array" aca="1" ref="D121" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A121&lt;&gt;""),$A$7:A121) &amp; "'!C:C"), $B121,
@@ -21044,9 +21047,9 @@
       </c>
     </row>
     <row r="122" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A122" s="28"/>
+      <c r="A122" s="73"/>
       <c r="B122" s="29" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C122" s="28">
         <f ca="1">IFERROR(
@@ -21067,11 +21070,11 @@
       </c>
     </row>
     <row r="123" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A123" s="24"/>
-      <c r="B123" s="25" t="s">
-        <v>96</v>
-      </c>
-      <c r="C123" s="24">
+      <c r="A123" s="28"/>
+      <c r="B123" s="29" t="s">
+        <v>97</v>
+      </c>
+      <c r="C123" s="28">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A123) &amp; "'!C:C"), B123),
    0
@@ -21090,11 +21093,11 @@
       </c>
     </row>
     <row r="124" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A124" s="38"/>
-      <c r="B124" s="43" t="s">
-        <v>95</v>
-      </c>
-      <c r="C124" s="28">
+      <c r="A124" s="24"/>
+      <c r="B124" s="25" t="s">
+        <v>96</v>
+      </c>
+      <c r="C124" s="24">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A124) &amp; "'!C:C"), B124),
    0
@@ -21113,9 +21116,9 @@
       </c>
     </row>
     <row r="125" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A125" s="28"/>
-      <c r="B125" s="29" t="s">
-        <v>94</v>
+      <c r="A125" s="38"/>
+      <c r="B125" s="43" t="s">
+        <v>95</v>
       </c>
       <c r="C125" s="28">
         <f ca="1">IFERROR(
@@ -21124,7 +21127,7 @@
 )</f>
         <v>0</v>
       </c>
-      <c r="D125" s="87" cm="1">
+      <c r="D125" s="73" cm="1">
         <f t="array" aca="1" ref="D125" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A125&lt;&gt;""),$A$7:A125) &amp; "'!C:C"), $B125,
@@ -21136,20 +21139,18 @@
       </c>
     </row>
     <row r="126" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A126" s="69" t="s">
-        <v>139</v>
-      </c>
-      <c r="B126" s="48" t="s">
-        <v>148</v>
-      </c>
-      <c r="C126" s="47">
+      <c r="A126" s="28"/>
+      <c r="B126" s="29" t="s">
+        <v>94</v>
+      </c>
+      <c r="C126" s="28">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A126) &amp; "'!C:C"), B126),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D126" s="88" cm="1">
+      <c r="D126" s="87" cm="1">
         <f t="array" aca="1" ref="D126" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A126&lt;&gt;""),$A$7:A126) &amp; "'!C:C"), $B126,
@@ -21161,18 +21162,20 @@
       </c>
     </row>
     <row r="127" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A127" s="31"/>
-      <c r="B127" s="30" t="s">
-        <v>149</v>
-      </c>
-      <c r="C127" s="28">
+      <c r="A127" s="69" t="s">
+        <v>139</v>
+      </c>
+      <c r="B127" s="48" t="s">
+        <v>148</v>
+      </c>
+      <c r="C127" s="47">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A127) &amp; "'!C:C"), B127),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D127" s="73" cm="1">
+      <c r="D127" s="88" cm="1">
         <f t="array" aca="1" ref="D127" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A127&lt;&gt;""),$A$7:A127) &amp; "'!C:C"), $B127,
@@ -21186,7 +21189,7 @@
     <row r="128" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A128" s="31"/>
       <c r="B128" s="30" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C128" s="28">
         <f ca="1">IFERROR(
@@ -21207,11 +21210,11 @@
       </c>
     </row>
     <row r="129" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A129" s="65"/>
-      <c r="B129" s="66" t="s">
-        <v>122</v>
-      </c>
-      <c r="C129" s="38">
+      <c r="A129" s="31"/>
+      <c r="B129" s="30" t="s">
+        <v>150</v>
+      </c>
+      <c r="C129" s="28">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A129) &amp; "'!C:C"), B129),
    0
@@ -21230,11 +21233,11 @@
       </c>
     </row>
     <row r="130" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A130" s="31"/>
-      <c r="B130" s="30" t="s">
-        <v>151</v>
-      </c>
-      <c r="C130" s="28">
+      <c r="A130" s="65"/>
+      <c r="B130" s="66" t="s">
+        <v>122</v>
+      </c>
+      <c r="C130" s="38">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A130) &amp; "'!C:C"), B130),
    0
@@ -21253,9 +21256,9 @@
       </c>
     </row>
     <row r="131" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A131" s="73"/>
-      <c r="B131" s="29" t="s">
-        <v>152</v>
+      <c r="A131" s="31"/>
+      <c r="B131" s="30" t="s">
+        <v>151</v>
       </c>
       <c r="C131" s="28">
         <f ca="1">IFERROR(
@@ -21264,7 +21267,7 @@
 )</f>
         <v>0</v>
       </c>
-      <c r="D131" s="87" cm="1">
+      <c r="D131" s="73" cm="1">
         <f t="array" aca="1" ref="D131" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A131&lt;&gt;""),$A$7:A131) &amp; "'!C:C"), $B131,
@@ -21276,20 +21279,18 @@
       </c>
     </row>
     <row r="132" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A132" s="69" t="s">
-        <v>140</v>
-      </c>
-      <c r="B132" s="48" t="s">
-        <v>141</v>
-      </c>
-      <c r="C132" s="47">
+      <c r="A132" s="73"/>
+      <c r="B132" s="29" t="s">
+        <v>152</v>
+      </c>
+      <c r="C132" s="28">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A132) &amp; "'!C:C"), B132),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D132" s="88" cm="1">
+      <c r="D132" s="87" cm="1">
         <f t="array" aca="1" ref="D132" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A132&lt;&gt;""),$A$7:A132) &amp; "'!C:C"), $B132,
@@ -21301,18 +21302,20 @@
       </c>
     </row>
     <row r="133" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A133" s="31"/>
-      <c r="B133" s="30" t="s">
-        <v>142</v>
-      </c>
-      <c r="C133" s="28">
+      <c r="A133" s="69" t="s">
+        <v>140</v>
+      </c>
+      <c r="B133" s="48" t="s">
+        <v>141</v>
+      </c>
+      <c r="C133" s="47">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A133) &amp; "'!C:C"), B133),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D133" s="73" cm="1">
+      <c r="D133" s="88" cm="1">
         <f t="array" aca="1" ref="D133" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A133&lt;&gt;""),$A$7:A133) &amp; "'!C:C"), $B133,
@@ -21326,7 +21329,7 @@
     <row r="134" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A134" s="31"/>
       <c r="B134" s="30" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C134" s="28">
         <f ca="1">IFERROR(
@@ -21347,11 +21350,11 @@
       </c>
     </row>
     <row r="135" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A135" s="65"/>
-      <c r="B135" s="66" t="s">
-        <v>144</v>
-      </c>
-      <c r="C135" s="38">
+      <c r="A135" s="31"/>
+      <c r="B135" s="30" t="s">
+        <v>143</v>
+      </c>
+      <c r="C135" s="28">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A135) &amp; "'!C:C"), B135),
    0
@@ -21370,11 +21373,11 @@
       </c>
     </row>
     <row r="136" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A136" s="31"/>
-      <c r="B136" s="30" t="s">
-        <v>145</v>
-      </c>
-      <c r="C136" s="28">
+      <c r="A136" s="65"/>
+      <c r="B136" s="66" t="s">
+        <v>144</v>
+      </c>
+      <c r="C136" s="38">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A136) &amp; "'!C:C"), B136),
    0
@@ -21393,9 +21396,9 @@
       </c>
     </row>
     <row r="137" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A137" s="73"/>
-      <c r="B137" s="29" t="s">
-        <v>146</v>
+      <c r="A137" s="31"/>
+      <c r="B137" s="30" t="s">
+        <v>145</v>
       </c>
       <c r="C137" s="28">
         <f ca="1">IFERROR(
@@ -21416,9 +21419,9 @@
       </c>
     </row>
     <row r="138" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A138" s="28"/>
+      <c r="A138" s="73"/>
       <c r="B138" s="29" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C138" s="28">
         <f ca="1">IFERROR(
@@ -21439,19 +21442,36 @@
       </c>
     </row>
     <row r="139" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A139" s="39"/>
-      <c r="B139" s="40"/>
-      <c r="C139" s="41"/>
-      <c r="D139" s="22"/>
+      <c r="A139" s="28"/>
+      <c r="B139" s="29" t="s">
+        <v>147</v>
+      </c>
+      <c r="C139" s="28">
+        <f ca="1">IFERROR(
+   COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A139) &amp; "'!C:C"), B139),
+   0
+)</f>
+        <v>0</v>
+      </c>
+      <c r="D139" s="73" cm="1">
+        <f t="array" aca="1" ref="D139" ca="1">IFERROR(
+  COUNTIFS(
+    INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A139&lt;&gt;""),$A$7:A139) &amp; "'!C:C"), $B139,
+    INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A139&lt;&gt;""),$A$7:A139) &amp; "'!E:E"), "&gt;=" &amp; ($B$3-6),
+    INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A139&lt;&gt;""),$A$7:A139) &amp; "'!E:E"), "&lt;=" &amp; $B$3
+  ),
+0)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="140" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A140" s="41"/>
-      <c r="B140" s="42"/>
+      <c r="A140" s="39"/>
+      <c r="B140" s="40"/>
       <c r="C140" s="41"/>
       <c r="D140" s="22"/>
     </row>
     <row r="141" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A141" s="39"/>
+      <c r="A141" s="41"/>
       <c r="B141" s="42"/>
       <c r="C141" s="41"/>
       <c r="D141" s="22"/>
@@ -21464,7 +21484,7 @@
     </row>
     <row r="143" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A143" s="39"/>
-      <c r="B143" s="40"/>
+      <c r="B143" s="42"/>
       <c r="C143" s="41"/>
       <c r="D143" s="22"/>
     </row>
@@ -21475,25 +21495,25 @@
       <c r="D144" s="22"/>
     </row>
     <row r="145" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A145" s="41"/>
+      <c r="A145" s="39"/>
       <c r="B145" s="40"/>
       <c r="C145" s="41"/>
       <c r="D145" s="22"/>
     </row>
     <row r="146" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A146" s="39"/>
+      <c r="A146" s="41"/>
       <c r="B146" s="40"/>
       <c r="C146" s="41"/>
       <c r="D146" s="22"/>
     </row>
     <row r="147" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A147" s="41"/>
+      <c r="A147" s="39"/>
       <c r="B147" s="40"/>
       <c r="C147" s="41"/>
       <c r="D147" s="22"/>
     </row>
     <row r="148" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A148" s="39"/>
+      <c r="A148" s="41"/>
       <c r="B148" s="40"/>
       <c r="C148" s="41"/>
       <c r="D148" s="22"/>
@@ -21553,13 +21573,13 @@
       <c r="D157" s="22"/>
     </row>
     <row r="158" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A158" s="41"/>
-      <c r="B158" s="42"/>
+      <c r="A158" s="39"/>
+      <c r="B158" s="40"/>
       <c r="C158" s="41"/>
       <c r="D158" s="22"/>
     </row>
     <row r="159" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A159" s="39"/>
+      <c r="A159" s="41"/>
       <c r="B159" s="42"/>
       <c r="C159" s="41"/>
       <c r="D159" s="22"/>
@@ -21572,7 +21592,7 @@
     </row>
     <row r="161" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A161" s="39"/>
-      <c r="B161" s="40"/>
+      <c r="B161" s="42"/>
       <c r="C161" s="41"/>
       <c r="D161" s="22"/>
     </row>
@@ -21583,25 +21603,25 @@
       <c r="D162" s="22"/>
     </row>
     <row r="163" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A163" s="41"/>
+      <c r="A163" s="39"/>
       <c r="B163" s="40"/>
       <c r="C163" s="41"/>
       <c r="D163" s="22"/>
     </row>
     <row r="164" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A164" s="39"/>
+      <c r="A164" s="41"/>
       <c r="B164" s="40"/>
       <c r="C164" s="41"/>
       <c r="D164" s="22"/>
     </row>
     <row r="165" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A165" s="41"/>
+      <c r="A165" s="39"/>
       <c r="B165" s="40"/>
       <c r="C165" s="41"/>
       <c r="D165" s="22"/>
     </row>
     <row r="166" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A166" s="39"/>
+      <c r="A166" s="41"/>
       <c r="B166" s="40"/>
       <c r="C166" s="41"/>
       <c r="D166" s="22"/>
@@ -21649,8 +21669,8 @@
       <c r="D173" s="22"/>
     </row>
     <row r="174" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A174" s="41"/>
-      <c r="B174" s="42"/>
+      <c r="A174" s="39"/>
+      <c r="B174" s="40"/>
       <c r="C174" s="41"/>
       <c r="D174" s="22"/>
     </row>
@@ -21799,9 +21819,9 @@
       <c r="D198" s="22"/>
     </row>
     <row r="199" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A199" s="23"/>
-      <c r="B199" s="21"/>
-      <c r="C199" s="21"/>
+      <c r="A199" s="41"/>
+      <c r="B199" s="42"/>
+      <c r="C199" s="41"/>
       <c r="D199" s="22"/>
     </row>
     <row r="200" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
@@ -22012,6 +22032,7 @@
       <c r="A234" s="23"/>
       <c r="B234" s="21"/>
       <c r="C234" s="21"/>
+      <c r="D234" s="22"/>
     </row>
     <row r="235" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A235" s="23"/>
@@ -22029,7 +22050,7 @@
       <c r="C237" s="21"/>
     </row>
     <row r="238" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A238" s="21"/>
+      <c r="A238" s="23"/>
       <c r="B238" s="21"/>
       <c r="C238" s="21"/>
     </row>
@@ -22121,6 +22142,7 @@
     <row r="256" spans="1:3" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A256" s="21"/>
       <c r="B256" s="21"/>
+      <c r="C256" s="21"/>
     </row>
     <row r="257" spans="1:2" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A257" s="21"/>
@@ -22385,6 +22407,10 @@
     <row r="322" spans="1:2" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A322" s="21"/>
       <c r="B322" s="21"/>
+    </row>
+    <row r="323" spans="1:2" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A323" s="21"/>
+      <c r="B323" s="21"/>
     </row>
   </sheetData>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
@@ -22394,7 +22420,7 @@
   </headerFooter>
   <rowBreaks count="2" manualBreakCount="2">
     <brk id="12" max="3" man="1"/>
-    <brk id="119" max="3" man="1"/>
+    <brk id="120" max="3" man="1"/>
   </rowBreaks>
   <legacyDrawingHF r:id="rId2"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update Body Motions spreadsheet with new content
</commit_message>
<xml_diff>
--- a/Month YEAR - Body Motions.xlsx
+++ b/Month YEAR - Body Motions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10517"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10525"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andyayas/VALD Automator/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E30D2D9-CAAF-2D48-BD93-DF30F377277F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1ADDFA9-9865-FC40-9242-BD5A611C24E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="REPORT 2" sheetId="10" r:id="rId1"/>
@@ -35,8 +35,8 @@
     <sheet name="Tabuk" sheetId="20" r:id="rId20"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">REPORT!$B$1:$B$362</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">REPORT!$A$1:$D$216</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">REPORT!$B$1:$B$363</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">REPORT!$A$1:$D$217</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'REPORT 2'!$A$1:$G$14</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'REPORT 2'!$1:$6</definedName>
   </definedNames>
@@ -83,7 +83,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="211">
   <si>
     <t>REPORT DATE:</t>
   </si>
@@ -719,6 +719,9 @@
   </si>
   <si>
     <t>Amal Al-Fahat Ghazi Al-Ruwaili</t>
+  </si>
+  <si>
+    <t>Wyssal Ben Dhieb</t>
   </si>
 </sst>
 </file>
@@ -1459,17 +1462,17 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -18306,7 +18309,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C7051E0-986F-8244-A07B-F9D8BD0E96B4}">
-  <dimension ref="A1:W362"/>
+  <dimension ref="A1:W363"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="50.83203125" defaultRowHeight="50" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="42.83203125" style="1" customWidth="1"/>
@@ -19619,7 +19622,7 @@
 )</f>
         <v>0</v>
       </c>
-      <c r="D59" s="112" cm="1">
+      <c r="D59" s="110" cm="1">
         <f t="array" aca="1" ref="D59" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A59&lt;&gt;""),$A$7:A59) &amp; "'!C:C"), $B59,
@@ -19644,7 +19647,7 @@
 )</f>
         <v>0</v>
       </c>
-      <c r="D60" s="111" cm="1">
+      <c r="D60" s="109" cm="1">
         <f t="array" aca="1" ref="D60" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A60&lt;&gt;""),$A$7:A60) &amp; "'!C:C"), $B60,
@@ -21173,7 +21176,7 @@
     <row r="123" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A123" s="24"/>
       <c r="B123" s="29" t="s">
-        <v>102</v>
+        <v>210</v>
       </c>
       <c r="C123" s="28">
         <f ca="1">IFERROR(
@@ -21194,9 +21197,9 @@
       </c>
     </row>
     <row r="124" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A124" s="73"/>
+      <c r="A124" s="24"/>
       <c r="B124" s="29" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C124" s="28">
         <f ca="1">IFERROR(
@@ -21217,9 +21220,9 @@
       </c>
     </row>
     <row r="125" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A125" s="28"/>
+      <c r="A125" s="73"/>
       <c r="B125" s="29" t="s">
-        <v>199</v>
+        <v>103</v>
       </c>
       <c r="C125" s="28">
         <f ca="1">IFERROR(
@@ -21242,7 +21245,7 @@
     <row r="126" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A126" s="28"/>
       <c r="B126" s="29" t="s">
-        <v>104</v>
+        <v>199</v>
       </c>
       <c r="C126" s="28">
         <f ca="1">IFERROR(
@@ -21265,7 +21268,7 @@
     <row r="127" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A127" s="28"/>
       <c r="B127" s="29" t="s">
-        <v>200</v>
+        <v>104</v>
       </c>
       <c r="C127" s="28">
         <f ca="1">IFERROR(
@@ -21286,18 +21289,18 @@
       </c>
     </row>
     <row r="128" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A128" s="80"/>
-      <c r="B128" s="75" t="s">
-        <v>159</v>
-      </c>
-      <c r="C128" s="80">
+      <c r="A128" s="28"/>
+      <c r="B128" s="29" t="s">
+        <v>200</v>
+      </c>
+      <c r="C128" s="28">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A128) &amp; "'!C:C"), B128),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D128" s="87" cm="1">
+      <c r="D128" s="73" cm="1">
         <f t="array" aca="1" ref="D128" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A128&lt;&gt;""),$A$7:A128) &amp; "'!C:C"), $B128,
@@ -21309,20 +21312,18 @@
       </c>
     </row>
     <row r="129" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A129" s="69" t="s">
-        <v>208</v>
-      </c>
-      <c r="B129" s="48" t="s">
-        <v>209</v>
-      </c>
-      <c r="C129" s="47">
+      <c r="A129" s="80"/>
+      <c r="B129" s="75" t="s">
+        <v>159</v>
+      </c>
+      <c r="C129" s="80">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A129) &amp; "'!C:C"), B129),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D129" s="88" cm="1">
+      <c r="D129" s="87" cm="1">
         <f t="array" aca="1" ref="D129" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A129&lt;&gt;""),$A$7:A129) &amp; "'!C:C"), $B129,
@@ -21334,18 +21335,20 @@
       </c>
     </row>
     <row r="130" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A130" s="31"/>
-      <c r="B130" s="30" t="s">
-        <v>101</v>
-      </c>
-      <c r="C130" s="28">
+      <c r="A130" s="69" t="s">
+        <v>208</v>
+      </c>
+      <c r="B130" s="48" t="s">
+        <v>209</v>
+      </c>
+      <c r="C130" s="47">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A130) &amp; "'!C:C"), B130),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D130" s="73" cm="1">
+      <c r="D130" s="88" cm="1">
         <f t="array" aca="1" ref="D130" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A130&lt;&gt;""),$A$7:A130) &amp; "'!C:C"), $B130,
@@ -21359,7 +21362,7 @@
     <row r="131" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A131" s="31"/>
       <c r="B131" s="30" t="s">
-        <v>30</v>
+        <v>101</v>
       </c>
       <c r="C131" s="28">
         <f ca="1">IFERROR(
@@ -21380,11 +21383,11 @@
       </c>
     </row>
     <row r="132" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A132" s="65"/>
-      <c r="B132" s="66" t="s">
-        <v>135</v>
-      </c>
-      <c r="C132" s="38">
+      <c r="A132" s="31"/>
+      <c r="B132" s="30" t="s">
+        <v>30</v>
+      </c>
+      <c r="C132" s="28">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A132) &amp; "'!C:C"), B132),
    0
@@ -21403,18 +21406,18 @@
       </c>
     </row>
     <row r="133" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A133" s="81"/>
-      <c r="B133" s="85" t="s">
-        <v>131</v>
-      </c>
-      <c r="C133" s="80">
+      <c r="A133" s="65"/>
+      <c r="B133" s="66" t="s">
+        <v>135</v>
+      </c>
+      <c r="C133" s="38">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A133) &amp; "'!C:C"), B133),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D133" s="112" cm="1">
+      <c r="D133" s="73" cm="1">
         <f t="array" aca="1" ref="D133" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A133&lt;&gt;""),$A$7:A133) &amp; "'!C:C"), $B133,
@@ -21426,20 +21429,18 @@
       </c>
     </row>
     <row r="134" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A134" s="24" t="s">
-        <v>90</v>
-      </c>
-      <c r="B134" s="25" t="s">
-        <v>111</v>
-      </c>
-      <c r="C134" s="24">
+      <c r="A134" s="81"/>
+      <c r="B134" s="85" t="s">
+        <v>131</v>
+      </c>
+      <c r="C134" s="80">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A134) &amp; "'!C:C"), B134),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D134" s="111" cm="1">
+      <c r="D134" s="110" cm="1">
         <f t="array" aca="1" ref="D134" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A134&lt;&gt;""),$A$7:A134) &amp; "'!C:C"), $B134,
@@ -21451,18 +21452,20 @@
       </c>
     </row>
     <row r="135" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A135" s="28"/>
-      <c r="B135" s="29" t="s">
-        <v>112</v>
-      </c>
-      <c r="C135" s="28">
+      <c r="A135" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="B135" s="25" t="s">
+        <v>111</v>
+      </c>
+      <c r="C135" s="24">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A135) &amp; "'!C:C"), B135),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D135" s="73" cm="1">
+      <c r="D135" s="109" cm="1">
         <f t="array" aca="1" ref="D135" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A135&lt;&gt;""),$A$7:A135) &amp; "'!C:C"), $B135,
@@ -21476,7 +21479,7 @@
     <row r="136" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A136" s="28"/>
       <c r="B136" s="29" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C136" s="28">
         <f ca="1">IFERROR(
@@ -21499,7 +21502,7 @@
     <row r="137" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A137" s="28"/>
       <c r="B137" s="29" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C137" s="28">
         <f ca="1">IFERROR(
@@ -21522,7 +21525,7 @@
     <row r="138" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A138" s="28"/>
       <c r="B138" s="29" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C138" s="28">
         <f ca="1">IFERROR(
@@ -21545,7 +21548,7 @@
     <row r="139" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A139" s="28"/>
       <c r="B139" s="29" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C139" s="28">
         <f ca="1">IFERROR(
@@ -21568,7 +21571,7 @@
     <row r="140" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A140" s="28"/>
       <c r="B140" s="29" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C140" s="28">
         <f ca="1">IFERROR(
@@ -21591,7 +21594,7 @@
     <row r="141" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A141" s="28"/>
       <c r="B141" s="29" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C141" s="28">
         <f ca="1">IFERROR(
@@ -21614,7 +21617,7 @@
     <row r="142" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A142" s="28"/>
       <c r="B142" s="29" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="C142" s="28">
         <f ca="1">IFERROR(
@@ -21637,7 +21640,7 @@
     <row r="143" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A143" s="28"/>
       <c r="B143" s="29" t="s">
-        <v>153</v>
+        <v>115</v>
       </c>
       <c r="C143" s="28">
         <f ca="1">IFERROR(
@@ -21658,9 +21661,9 @@
       </c>
     </row>
     <row r="144" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A144" s="31"/>
-      <c r="B144" s="30" t="s">
-        <v>160</v>
+      <c r="A144" s="28"/>
+      <c r="B144" s="29" t="s">
+        <v>153</v>
       </c>
       <c r="C144" s="28">
         <f ca="1">IFERROR(
@@ -21683,7 +21686,7 @@
     <row r="145" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A145" s="31"/>
       <c r="B145" s="30" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="C145" s="28">
         <f ca="1">IFERROR(
@@ -21704,18 +21707,18 @@
       </c>
     </row>
     <row r="146" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A146" s="79"/>
-      <c r="B146" s="78" t="s">
-        <v>201</v>
-      </c>
-      <c r="C146" s="77">
+      <c r="A146" s="31"/>
+      <c r="B146" s="30" t="s">
+        <v>167</v>
+      </c>
+      <c r="C146" s="28">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A146) &amp; "'!C:C"), B146),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D146" s="87" cm="1">
+      <c r="D146" s="73" cm="1">
         <f t="array" aca="1" ref="D146" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A146&lt;&gt;""),$A$7:A146) &amp; "'!C:C"), $B146,
@@ -21727,20 +21730,18 @@
       </c>
     </row>
     <row r="147" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A147" s="24" t="s">
-        <v>89</v>
-      </c>
-      <c r="B147" s="25" t="s">
-        <v>105</v>
-      </c>
-      <c r="C147" s="24">
+      <c r="A147" s="79"/>
+      <c r="B147" s="78" t="s">
+        <v>201</v>
+      </c>
+      <c r="C147" s="77">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A147) &amp; "'!C:C"), B147),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D147" s="88" cm="1">
+      <c r="D147" s="87" cm="1">
         <f t="array" aca="1" ref="D147" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A147&lt;&gt;""),$A$7:A147) &amp; "'!C:C"), $B147,
@@ -21752,18 +21753,20 @@
       </c>
     </row>
     <row r="148" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A148" s="28"/>
-      <c r="B148" s="29" t="s">
-        <v>106</v>
-      </c>
-      <c r="C148" s="28">
+      <c r="A148" s="24" t="s">
+        <v>89</v>
+      </c>
+      <c r="B148" s="25" t="s">
+        <v>105</v>
+      </c>
+      <c r="C148" s="24">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A148) &amp; "'!C:C"), B148),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D148" s="73" cm="1">
+      <c r="D148" s="88" cm="1">
         <f t="array" aca="1" ref="D148" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A148&lt;&gt;""),$A$7:A148) &amp; "'!C:C"), $B148,
@@ -21777,7 +21780,7 @@
     <row r="149" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A149" s="28"/>
       <c r="B149" s="29" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C149" s="28">
         <f ca="1">IFERROR(
@@ -21800,7 +21803,7 @@
     <row r="150" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A150" s="28"/>
       <c r="B150" s="29" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C150" s="28">
         <f ca="1">IFERROR(
@@ -21823,7 +21826,7 @@
     <row r="151" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A151" s="28"/>
       <c r="B151" s="29" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C151" s="28">
         <f ca="1">IFERROR(
@@ -21846,7 +21849,7 @@
     <row r="152" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A152" s="28"/>
       <c r="B152" s="29" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C152" s="28">
         <f ca="1">IFERROR(
@@ -21867,18 +21870,18 @@
       </c>
     </row>
     <row r="153" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A153" s="76"/>
-      <c r="B153" s="75" t="s">
-        <v>162</v>
-      </c>
-      <c r="C153" s="74">
+      <c r="A153" s="28"/>
+      <c r="B153" s="29" t="s">
+        <v>110</v>
+      </c>
+      <c r="C153" s="28">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A153) &amp; "'!C:C"), B153),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D153" s="87" cm="1">
+      <c r="D153" s="73" cm="1">
         <f t="array" aca="1" ref="D153" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A153&lt;&gt;""),$A$7:A153) &amp; "'!C:C"), $B153,
@@ -21890,20 +21893,18 @@
       </c>
     </row>
     <row r="154" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A154" s="69" t="s">
-        <v>87</v>
-      </c>
-      <c r="B154" s="66" t="s">
-        <v>94</v>
-      </c>
-      <c r="C154" s="47">
+      <c r="A154" s="76"/>
+      <c r="B154" s="75" t="s">
+        <v>162</v>
+      </c>
+      <c r="C154" s="74">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A154) &amp; "'!C:C"), B154),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D154" s="88" cm="1">
+      <c r="D154" s="87" cm="1">
         <f t="array" aca="1" ref="D154" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A154&lt;&gt;""),$A$7:A154) &amp; "'!C:C"), $B154,
@@ -21915,18 +21916,20 @@
       </c>
     </row>
     <row r="155" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A155" s="73"/>
-      <c r="B155" s="29" t="s">
-        <v>96</v>
-      </c>
-      <c r="C155" s="28">
+      <c r="A155" s="69" t="s">
+        <v>87</v>
+      </c>
+      <c r="B155" s="66" t="s">
+        <v>94</v>
+      </c>
+      <c r="C155" s="47">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A155) &amp; "'!C:C"), B155),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D155" s="73" cm="1">
+      <c r="D155" s="88" cm="1">
         <f t="array" aca="1" ref="D155" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A155&lt;&gt;""),$A$7:A155) &amp; "'!C:C"), $B155,
@@ -21940,7 +21943,7 @@
     <row r="156" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A156" s="73"/>
       <c r="B156" s="29" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C156" s="28">
         <f ca="1">IFERROR(
@@ -21963,7 +21966,7 @@
     <row r="157" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A157" s="73"/>
       <c r="B157" s="29" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C157" s="28">
         <f ca="1">IFERROR(
@@ -21986,7 +21989,7 @@
     <row r="158" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A158" s="73"/>
       <c r="B158" s="29" t="s">
-        <v>202</v>
+        <v>98</v>
       </c>
       <c r="C158" s="28">
         <f ca="1">IFERROR(
@@ -22007,9 +22010,9 @@
       </c>
     </row>
     <row r="159" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A159" s="28"/>
+      <c r="A159" s="73"/>
       <c r="B159" s="29" t="s">
-        <v>99</v>
+        <v>202</v>
       </c>
       <c r="C159" s="28">
         <f ca="1">IFERROR(
@@ -22030,9 +22033,9 @@
       </c>
     </row>
     <row r="160" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A160" s="24"/>
-      <c r="B160" s="25" t="s">
-        <v>203</v>
+      <c r="A160" s="28"/>
+      <c r="B160" s="29" t="s">
+        <v>99</v>
       </c>
       <c r="C160" s="28">
         <f ca="1">IFERROR(
@@ -22055,7 +22058,7 @@
     <row r="161" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A161" s="24"/>
       <c r="B161" s="25" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C161" s="28">
         <f ca="1">IFERROR(
@@ -22078,9 +22081,9 @@
     <row r="162" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A162" s="24"/>
       <c r="B162" s="25" t="s">
-        <v>205</v>
-      </c>
-      <c r="C162" s="24">
+        <v>204</v>
+      </c>
+      <c r="C162" s="28">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A162) &amp; "'!C:C"), B162),
    0
@@ -22099,11 +22102,11 @@
       </c>
     </row>
     <row r="163" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A163" s="38"/>
-      <c r="B163" s="43" t="s">
-        <v>95</v>
-      </c>
-      <c r="C163" s="28">
+      <c r="A163" s="24"/>
+      <c r="B163" s="25" t="s">
+        <v>205</v>
+      </c>
+      <c r="C163" s="24">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A163) &amp; "'!C:C"), B163),
    0
@@ -22122,9 +22125,9 @@
       </c>
     </row>
     <row r="164" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A164" s="28"/>
-      <c r="B164" s="29" t="s">
-        <v>206</v>
+      <c r="A164" s="38"/>
+      <c r="B164" s="43" t="s">
+        <v>95</v>
       </c>
       <c r="C164" s="28">
         <f ca="1">IFERROR(
@@ -22133,7 +22136,7 @@
 )</f>
         <v>0</v>
       </c>
-      <c r="D164" s="87" cm="1">
+      <c r="D164" s="73" cm="1">
         <f t="array" aca="1" ref="D164" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A164&lt;&gt;""),$A$7:A164) &amp; "'!C:C"), $B164,
@@ -22145,20 +22148,18 @@
       </c>
     </row>
     <row r="165" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A165" s="69" t="s">
-        <v>139</v>
-      </c>
-      <c r="B165" s="48" t="s">
-        <v>152</v>
-      </c>
-      <c r="C165" s="47">
+      <c r="A165" s="28"/>
+      <c r="B165" s="29" t="s">
+        <v>206</v>
+      </c>
+      <c r="C165" s="28">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A165) &amp; "'!C:C"), B165),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D165" s="88" cm="1">
+      <c r="D165" s="87" cm="1">
         <f t="array" aca="1" ref="D165" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A165&lt;&gt;""),$A$7:A165) &amp; "'!C:C"), $B165,
@@ -22170,18 +22171,20 @@
       </c>
     </row>
     <row r="166" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A166" s="31"/>
-      <c r="B166" s="30" t="s">
-        <v>151</v>
-      </c>
-      <c r="C166" s="28">
+      <c r="A166" s="69" t="s">
+        <v>139</v>
+      </c>
+      <c r="B166" s="48" t="s">
+        <v>152</v>
+      </c>
+      <c r="C166" s="47">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A166) &amp; "'!C:C"), B166),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D166" s="73" cm="1">
+      <c r="D166" s="88" cm="1">
         <f t="array" aca="1" ref="D166" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A166&lt;&gt;""),$A$7:A166) &amp; "'!C:C"), $B166,
@@ -22195,7 +22198,7 @@
     <row r="167" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A167" s="31"/>
       <c r="B167" s="30" t="s">
-        <v>122</v>
+        <v>151</v>
       </c>
       <c r="C167" s="28">
         <f ca="1">IFERROR(
@@ -22216,11 +22219,11 @@
       </c>
     </row>
     <row r="168" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A168" s="65"/>
-      <c r="B168" s="66" t="s">
-        <v>150</v>
-      </c>
-      <c r="C168" s="38">
+      <c r="A168" s="31"/>
+      <c r="B168" s="30" t="s">
+        <v>122</v>
+      </c>
+      <c r="C168" s="28">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A168) &amp; "'!C:C"), B168),
    0
@@ -22239,11 +22242,11 @@
       </c>
     </row>
     <row r="169" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A169" s="31"/>
-      <c r="B169" s="30" t="s">
-        <v>149</v>
-      </c>
-      <c r="C169" s="28">
+      <c r="A169" s="65"/>
+      <c r="B169" s="66" t="s">
+        <v>150</v>
+      </c>
+      <c r="C169" s="38">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A169) &amp; "'!C:C"), B169),
    0
@@ -22262,9 +22265,9 @@
       </c>
     </row>
     <row r="170" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A170" s="73"/>
-      <c r="B170" s="29" t="s">
-        <v>148</v>
+      <c r="A170" s="31"/>
+      <c r="B170" s="30" t="s">
+        <v>149</v>
       </c>
       <c r="C170" s="28">
         <f ca="1">IFERROR(
@@ -22273,7 +22276,7 @@
 )</f>
         <v>0</v>
       </c>
-      <c r="D170" s="87" cm="1">
+      <c r="D170" s="73" cm="1">
         <f t="array" aca="1" ref="D170" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A170&lt;&gt;""),$A$7:A170) &amp; "'!C:C"), $B170,
@@ -22285,20 +22288,18 @@
       </c>
     </row>
     <row r="171" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A171" s="69" t="s">
-        <v>140</v>
-      </c>
-      <c r="B171" s="48" t="s">
-        <v>147</v>
-      </c>
-      <c r="C171" s="47">
+      <c r="A171" s="73"/>
+      <c r="B171" s="29" t="s">
+        <v>148</v>
+      </c>
+      <c r="C171" s="28">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A171) &amp; "'!C:C"), B171),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D171" s="88" cm="1">
+      <c r="D171" s="87" cm="1">
         <f t="array" aca="1" ref="D171" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A171&lt;&gt;""),$A$7:A171) &amp; "'!C:C"), $B171,
@@ -22310,18 +22311,20 @@
       </c>
     </row>
     <row r="172" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A172" s="31"/>
-      <c r="B172" s="30" t="s">
-        <v>146</v>
-      </c>
-      <c r="C172" s="28">
+      <c r="A172" s="69" t="s">
+        <v>140</v>
+      </c>
+      <c r="B172" s="48" t="s">
+        <v>147</v>
+      </c>
+      <c r="C172" s="47">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A172) &amp; "'!C:C"), B172),
    0
 )</f>
         <v>0</v>
       </c>
-      <c r="D172" s="73" cm="1">
+      <c r="D172" s="88" cm="1">
         <f t="array" aca="1" ref="D172" ca="1">IFERROR(
   COUNTIFS(
     INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A172&lt;&gt;""),$A$7:A172) &amp; "'!C:C"), $B172,
@@ -22335,7 +22338,7 @@
     <row r="173" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A173" s="31"/>
       <c r="B173" s="30" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C173" s="28">
         <f ca="1">IFERROR(
@@ -22356,9 +22359,9 @@
       </c>
     </row>
     <row r="174" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A174" s="65"/>
-      <c r="B174" s="66" t="s">
-        <v>144</v>
+      <c r="A174" s="31"/>
+      <c r="B174" s="30" t="s">
+        <v>145</v>
       </c>
       <c r="C174" s="28">
         <f ca="1">IFERROR(
@@ -22381,9 +22384,9 @@
     <row r="175" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A175" s="65"/>
       <c r="B175" s="66" t="s">
-        <v>143</v>
-      </c>
-      <c r="C175" s="38">
+        <v>144</v>
+      </c>
+      <c r="C175" s="28">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A175) &amp; "'!C:C"), B175),
    0
@@ -22402,11 +22405,11 @@
       </c>
     </row>
     <row r="176" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A176" s="31"/>
-      <c r="B176" s="30" t="s">
-        <v>142</v>
-      </c>
-      <c r="C176" s="28">
+      <c r="A176" s="65"/>
+      <c r="B176" s="66" t="s">
+        <v>143</v>
+      </c>
+      <c r="C176" s="38">
         <f ca="1">IFERROR(
    COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A176) &amp; "'!C:C"), B176),
    0
@@ -22425,9 +22428,9 @@
       </c>
     </row>
     <row r="177" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A177" s="73"/>
-      <c r="B177" s="29" t="s">
-        <v>141</v>
+      <c r="A177" s="31"/>
+      <c r="B177" s="30" t="s">
+        <v>142</v>
       </c>
       <c r="C177" s="28">
         <f ca="1">IFERROR(
@@ -22448,9 +22451,9 @@
       </c>
     </row>
     <row r="178" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A178" s="28"/>
+      <c r="A178" s="73"/>
       <c r="B178" s="29" t="s">
-        <v>207</v>
+        <v>141</v>
       </c>
       <c r="C178" s="28">
         <f ca="1">IFERROR(
@@ -22471,19 +22474,36 @@
       </c>
     </row>
     <row r="179" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A179" s="39"/>
-      <c r="B179" s="40"/>
-      <c r="C179" s="41"/>
-      <c r="D179" s="22"/>
+      <c r="A179" s="28"/>
+      <c r="B179" s="29" t="s">
+        <v>207</v>
+      </c>
+      <c r="C179" s="28">
+        <f ca="1">IFERROR(
+   COUNTIF(INDIRECT("'" &amp; LOOKUP("zzz",$A$7:A179) &amp; "'!C:C"), B179),
+   0
+)</f>
+        <v>0</v>
+      </c>
+      <c r="D179" s="73" cm="1">
+        <f t="array" aca="1" ref="D179" ca="1">IFERROR(
+  COUNTIFS(
+    INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A179&lt;&gt;""),$A$7:A179) &amp; "'!C:C"), $B179,
+    INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A179&lt;&gt;""),$A$7:A179) &amp; "'!E:E"), "&gt;=" &amp; ($B$3-6),
+    INDIRECT("'" &amp; LOOKUP(2,1/($A$7:A179&lt;&gt;""),$A$7:A179) &amp; "'!E:E"), "&lt;=" &amp; $B$3
+  ),
+0)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="180" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A180" s="41"/>
-      <c r="B180" s="42"/>
+      <c r="A180" s="39"/>
+      <c r="B180" s="40"/>
       <c r="C180" s="41"/>
       <c r="D180" s="22"/>
     </row>
     <row r="181" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A181" s="39"/>
+      <c r="A181" s="41"/>
       <c r="B181" s="42"/>
       <c r="C181" s="41"/>
       <c r="D181" s="22"/>
@@ -22496,7 +22516,7 @@
     </row>
     <row r="183" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A183" s="39"/>
-      <c r="B183" s="40"/>
+      <c r="B183" s="42"/>
       <c r="C183" s="41"/>
       <c r="D183" s="22"/>
     </row>
@@ -22507,25 +22527,25 @@
       <c r="D184" s="22"/>
     </row>
     <row r="185" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A185" s="41"/>
+      <c r="A185" s="39"/>
       <c r="B185" s="40"/>
       <c r="C185" s="41"/>
       <c r="D185" s="22"/>
     </row>
     <row r="186" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A186" s="39"/>
+      <c r="A186" s="41"/>
       <c r="B186" s="40"/>
       <c r="C186" s="41"/>
       <c r="D186" s="22"/>
     </row>
     <row r="187" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A187" s="41"/>
+      <c r="A187" s="39"/>
       <c r="B187" s="40"/>
       <c r="C187" s="41"/>
       <c r="D187" s="22"/>
     </row>
     <row r="188" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A188" s="39"/>
+      <c r="A188" s="41"/>
       <c r="B188" s="40"/>
       <c r="C188" s="41"/>
       <c r="D188" s="22"/>
@@ -22585,13 +22605,13 @@
       <c r="D197" s="22"/>
     </row>
     <row r="198" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A198" s="41"/>
-      <c r="B198" s="42"/>
+      <c r="A198" s="39"/>
+      <c r="B198" s="40"/>
       <c r="C198" s="41"/>
       <c r="D198" s="22"/>
     </row>
     <row r="199" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A199" s="39"/>
+      <c r="A199" s="41"/>
       <c r="B199" s="42"/>
       <c r="C199" s="41"/>
       <c r="D199" s="22"/>
@@ -22604,7 +22624,7 @@
     </row>
     <row r="201" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A201" s="39"/>
-      <c r="B201" s="40"/>
+      <c r="B201" s="42"/>
       <c r="C201" s="41"/>
       <c r="D201" s="22"/>
     </row>
@@ -22615,25 +22635,25 @@
       <c r="D202" s="22"/>
     </row>
     <row r="203" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A203" s="41"/>
+      <c r="A203" s="39"/>
       <c r="B203" s="40"/>
       <c r="C203" s="41"/>
       <c r="D203" s="22"/>
     </row>
     <row r="204" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A204" s="39"/>
+      <c r="A204" s="41"/>
       <c r="B204" s="40"/>
       <c r="C204" s="41"/>
       <c r="D204" s="22"/>
     </row>
     <row r="205" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A205" s="41"/>
+      <c r="A205" s="39"/>
       <c r="B205" s="40"/>
       <c r="C205" s="41"/>
       <c r="D205" s="22"/>
     </row>
     <row r="206" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A206" s="39"/>
+      <c r="A206" s="41"/>
       <c r="B206" s="40"/>
       <c r="C206" s="41"/>
       <c r="D206" s="22"/>
@@ -22681,8 +22701,8 @@
       <c r="D213" s="22"/>
     </row>
     <row r="214" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A214" s="41"/>
-      <c r="B214" s="42"/>
+      <c r="A214" s="39"/>
+      <c r="B214" s="40"/>
       <c r="C214" s="41"/>
       <c r="D214" s="22"/>
     </row>
@@ -22831,9 +22851,9 @@
       <c r="D238" s="22"/>
     </row>
     <row r="239" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A239" s="23"/>
-      <c r="B239" s="21"/>
-      <c r="C239" s="21"/>
+      <c r="A239" s="41"/>
+      <c r="B239" s="42"/>
+      <c r="C239" s="41"/>
       <c r="D239" s="22"/>
     </row>
     <row r="240" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
@@ -23044,6 +23064,7 @@
       <c r="A274" s="23"/>
       <c r="B274" s="21"/>
       <c r="C274" s="21"/>
+      <c r="D274" s="22"/>
     </row>
     <row r="275" spans="1:23" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A275" s="23"/>
@@ -23061,7 +23082,7 @@
       <c r="C277" s="21"/>
     </row>
     <row r="278" spans="1:23" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A278" s="21"/>
+      <c r="A278" s="23"/>
       <c r="B278" s="21"/>
       <c r="C278" s="21"/>
     </row>
@@ -23070,29 +23091,10 @@
       <c r="B279" s="21"/>
       <c r="C279" s="21"/>
     </row>
-    <row r="280" spans="1:23" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="280" spans="1:23" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A280" s="21"/>
       <c r="B280" s="21"/>
       <c r="C280" s="21"/>
-      <c r="E280" s="1"/>
-      <c r="F280" s="1"/>
-      <c r="G280" s="1"/>
-      <c r="H280" s="1"/>
-      <c r="I280" s="1"/>
-      <c r="J280" s="1"/>
-      <c r="K280" s="1"/>
-      <c r="L280" s="1"/>
-      <c r="M280" s="1"/>
-      <c r="N280" s="1"/>
-      <c r="O280" s="1"/>
-      <c r="P280" s="1"/>
-      <c r="Q280" s="1"/>
-      <c r="R280" s="1"/>
-      <c r="S280" s="1"/>
-      <c r="T280" s="1"/>
-      <c r="U280" s="1"/>
-      <c r="V280" s="1"/>
-      <c r="W280" s="1"/>
     </row>
     <row r="281" spans="1:23" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A281" s="21"/>
@@ -23454,9 +23456,29 @@
       <c r="V295" s="1"/>
       <c r="W295" s="1"/>
     </row>
-    <row r="296" spans="1:23" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="296" spans="1:23" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A296" s="21"/>
       <c r="B296" s="21"/>
+      <c r="C296" s="21"/>
+      <c r="E296" s="1"/>
+      <c r="F296" s="1"/>
+      <c r="G296" s="1"/>
+      <c r="H296" s="1"/>
+      <c r="I296" s="1"/>
+      <c r="J296" s="1"/>
+      <c r="K296" s="1"/>
+      <c r="L296" s="1"/>
+      <c r="M296" s="1"/>
+      <c r="N296" s="1"/>
+      <c r="O296" s="1"/>
+      <c r="P296" s="1"/>
+      <c r="Q296" s="1"/>
+      <c r="R296" s="1"/>
+      <c r="S296" s="1"/>
+      <c r="T296" s="1"/>
+      <c r="U296" s="1"/>
+      <c r="V296" s="1"/>
+      <c r="W296" s="1"/>
     </row>
     <row r="297" spans="1:23" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A297" s="21"/>
@@ -23721,6 +23743,10 @@
     <row r="362" spans="1:2" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A362" s="21"/>
       <c r="B362" s="21"/>
+    </row>
+    <row r="363" spans="1:2" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A363" s="21"/>
+      <c r="B363" s="21"/>
     </row>
   </sheetData>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
@@ -23730,7 +23756,7 @@
   </headerFooter>
   <rowBreaks count="2" manualBreakCount="2">
     <brk id="19" max="3" man="1"/>
-    <brk id="153" max="3" man="1"/>
+    <brk id="154" max="3" man="1"/>
   </rowBreaks>
   <legacyDrawingHF r:id="rId2"/>
 </worksheet>
@@ -27176,9 +27202,9 @@
       <c r="C31" s="98"/>
       <c r="D31" s="104"/>
       <c r="E31" s="104"/>
-      <c r="F31" s="109"/>
-      <c r="G31" s="110"/>
-      <c r="H31" s="110"/>
+      <c r="F31" s="111"/>
+      <c r="G31" s="112"/>
+      <c r="H31" s="112"/>
     </row>
     <row r="32" spans="1:8" s="106" customFormat="1" ht="62" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A32" s="102"/>

</xml_diff>

<commit_message>
fix: update Body Motions and Payment spreadsheets with latest data
</commit_message>
<xml_diff>
--- a/Month YEAR - Body Motions.xlsx
+++ b/Month YEAR - Body Motions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andyayas/VALD Automator/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A6271E9-60DA-0745-9369-F76B2458B77E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A58FCDD-2E0D-CB49-B375-4ECEE175669B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="469" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="213">
   <si>
     <t>REPORT DATE:</t>
   </si>
@@ -701,6 +701,9 @@
   </si>
   <si>
     <t>تاريخ ارسال الجدول</t>
+  </si>
+  <si>
+    <t>ALQ - Al Rayyan</t>
   </si>
 </sst>
 </file>
@@ -1731,7 +1734,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P76"/>
+  <dimension ref="A1:P77"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="60" style="1" customWidth="1"/>
@@ -1767,7 +1770,7 @@
         <v>1</v>
       </c>
       <c r="D3" s="89">
-        <f ca="1">SUM(C7:C25)</f>
+        <f ca="1">SUM(C7:C26)</f>
         <v>0</v>
       </c>
     </row>
@@ -1811,7 +1814,7 @@
         <v>10</v>
       </c>
       <c r="B7" s="37">
-        <f t="shared" ref="B7:B25" ca="1" si="0">IFERROR(COUNTIFS(INDIRECT("'" &amp; $A7 &amp; "'!E:E"), "&gt;=" &amp; $B$3-7, INDIRECT("'" &amp; $A7 &amp; "'!E:E"), "&lt;=" &amp; $B$3),0)</f>
+        <f t="shared" ref="B7:B26" ca="1" si="0">IFERROR(COUNTIFS(INDIRECT("'" &amp; $A7 &amp; "'!E:E"), "&gt;=" &amp; $B$3-7, INDIRECT("'" &amp; $A7 &amp; "'!E:E"), "&lt;=" &amp; $B$3),0)</f>
         <v>0</v>
       </c>
       <c r="C7" s="36">
@@ -2094,7 +2097,7 @@
     </row>
     <row r="21" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="58" t="s">
-        <v>24</v>
+        <v>212</v>
       </c>
       <c r="B21" s="37">
         <f t="shared" ca="1" si="0"/>
@@ -2105,14 +2108,14 @@
         <v>0</v>
       </c>
       <c r="D21" s="36">
-        <f ca="1">C21+29</f>
-        <v>29</v>
+        <f ca="1">C21+0</f>
+        <v>0</v>
       </c>
       <c r="E21" s="17"/>
     </row>
     <row r="22" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="31" t="s">
-        <v>25</v>
+      <c r="A22" s="58" t="s">
+        <v>24</v>
       </c>
       <c r="B22" s="37">
         <f t="shared" ca="1" si="0"/>
@@ -2123,14 +2126,14 @@
         <v>0</v>
       </c>
       <c r="D22" s="36">
-        <f ca="1">C22+20</f>
-        <v>20</v>
+        <f ca="1">C22+29</f>
+        <v>29</v>
       </c>
       <c r="E22" s="17"/>
     </row>
     <row r="23" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="57" t="s">
-        <v>26</v>
+      <c r="A23" s="31" t="s">
+        <v>25</v>
       </c>
       <c r="B23" s="37">
         <f t="shared" ca="1" si="0"/>
@@ -2141,14 +2144,14 @@
         <v>0</v>
       </c>
       <c r="D23" s="36">
-        <f ca="1">C23+48</f>
-        <v>48</v>
+        <f ca="1">C23+20</f>
+        <v>20</v>
       </c>
       <c r="E23" s="17"/>
     </row>
     <row r="24" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="31" t="s">
-        <v>27</v>
+      <c r="A24" s="57" t="s">
+        <v>26</v>
       </c>
       <c r="B24" s="37">
         <f t="shared" ca="1" si="0"/>
@@ -2159,14 +2162,14 @@
         <v>0</v>
       </c>
       <c r="D24" s="36">
-        <f ca="1">C24+16</f>
-        <v>16</v>
+        <f ca="1">C24+48</f>
+        <v>48</v>
       </c>
       <c r="E24" s="17"/>
     </row>
     <row r="25" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="57" t="s">
-        <v>28</v>
+      <c r="A25" s="31" t="s">
+        <v>27</v>
       </c>
       <c r="B25" s="37">
         <f t="shared" ca="1" si="0"/>
@@ -2177,16 +2180,27 @@
         <v>0</v>
       </c>
       <c r="D25" s="36">
-        <f ca="1">C25+11</f>
+        <f ca="1">C25+16</f>
+        <v>16</v>
+      </c>
+      <c r="E25" s="17"/>
+    </row>
+    <row r="26" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="57" t="s">
+        <v>28</v>
+      </c>
+      <c r="B26" s="37">
+        <f t="shared" ca="1" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="C26" s="36">
+        <f t="array" aca="1" ref="C26" ca="1">INDIRECT("'" &amp; A26 &amp; "'!D3")</f>
+        <v>0</v>
+      </c>
+      <c r="D26" s="36">
+        <f ca="1">C26+11</f>
         <v>11</v>
       </c>
-      <c r="E25" s="17"/>
-    </row>
-    <row r="26" spans="1:5" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="17"/>
-      <c r="B26" s="17"/>
-      <c r="C26" s="35"/>
-      <c r="D26" s="35"/>
       <c r="E26" s="17"/>
     </row>
     <row r="27" spans="1:5" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -2516,6 +2530,7 @@
       <c r="B73" s="17"/>
       <c r="C73" s="35"/>
       <c r="D73" s="35"/>
+      <c r="E73" s="17"/>
     </row>
     <row r="74" spans="1:5" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="17"/>
@@ -2534,6 +2549,12 @@
       <c r="B76" s="17"/>
       <c r="C76" s="35"/>
       <c r="D76" s="35"/>
+    </row>
+    <row r="77" spans="1:5" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A77" s="17"/>
+      <c r="B77" s="17"/>
+      <c r="C77" s="35"/>
+      <c r="D77" s="35"/>
     </row>
   </sheetData>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>

</xml_diff>